<commit_message>
Daily EOD data and reports for 2026-09-08
</commit_message>
<xml_diff>
--- a/asx_eod_output/Report_XLSX/Report_20260908.xlsx
+++ b/asx_eod_output/Report_XLSX/Report_20260908.xlsx
@@ -488,24 +488,24 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>1.9</v>
+        <v>1.92</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>-0.01</v>
+        <v>0.01</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>-0.52%</t>
+          <t>0.52%</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
         <v>153181</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>291043.9</v>
+        <v>294107.52</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>-1531.81</v>
+        <v>1531.81</v>
       </c>
     </row>
     <row r="5">
@@ -515,24 +515,24 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>2.455</v>
+        <v>2.44</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>0.015</v>
+        <v>0</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>0.61%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
         <v>70000</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>171850</v>
+        <v>170800</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>1050</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -623,14 +623,14 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>159.09</v>
+        <v>158.69</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>-2.45</v>
+        <v>-2.85</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>-1.52%</t>
+          <t>-1.76%</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
@@ -650,24 +650,24 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>0.975</v>
+        <v>0.96</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0</v>
+        <v>-0.015</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>-1.54%</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
         <v>10000</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>9750</v>
+        <v>9600</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>0</v>
+        <v>-150</v>
       </c>
     </row>
     <row r="11">
@@ -677,24 +677,24 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>172.01</v>
+        <v>174.8</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>-1.17</v>
+        <v>1.62</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>-0.68%</t>
+          <t>0.94%</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
         <v>4000</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>688040</v>
+        <v>699200</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>-4680</v>
+        <v>6480</v>
       </c>
     </row>
     <row r="12">
@@ -704,24 +704,24 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>0.285</v>
+        <v>0.27</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0.01</v>
+        <v>-0.005</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>3.64%</t>
+          <t>-1.82%</t>
         </is>
       </c>
       <c r="E12" s="3" t="n">
         <v>20000</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>5700</v>
+        <v>5400</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>200</v>
+        <v>-100</v>
       </c>
     </row>
     <row r="13">
@@ -731,24 +731,24 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>0</v>
+        <v>0.002</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>-0.002</v>
+        <v>0</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>-100.00%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="E13" s="3" t="n">
         <v>700000</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>0</v>
+        <v>1400</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>-1400</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -758,24 +758,24 @@
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>0.115</v>
+        <v>0.12</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>0</v>
+        <v>0.005</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>4.35%</t>
         </is>
       </c>
       <c r="E14" s="3" t="n">
         <v>9412</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>1082.38</v>
+        <v>1129.44</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>0</v>
+        <v>47.06</v>
       </c>
     </row>
     <row r="15">
@@ -785,24 +785,24 @@
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>0.096</v>
+        <v>0.095</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>0</v>
+        <v>-0.001</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>-1.04%</t>
         </is>
       </c>
       <c r="E15" s="3" t="n">
         <v>6000</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>576</v>
+        <v>570</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>0</v>
+        <v>-6</v>
       </c>
     </row>
     <row r="16">
@@ -812,14 +812,14 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>34.7</v>
+        <v>34.58</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>-0.32</v>
+        <v>-0.44</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>-0.91%</t>
+          <t>-1.26%</t>
         </is>
       </c>
       <c r="E16" s="3" t="n">
@@ -839,24 +839,24 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>32.25</v>
+        <v>32.3</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>-0.08</v>
+        <v>-0.03</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>-0.25%</t>
+          <t>-0.09%</t>
         </is>
       </c>
       <c r="E17" s="3" t="n">
         <v>1288</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>41538</v>
+        <v>41602.4</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>-103.04</v>
+        <v>-38.64</v>
       </c>
     </row>
     <row r="18">
@@ -870,10 +870,10 @@
       <c r="D18" s="5" t="inlineStr"/>
       <c r="E18" s="7" t="inlineStr"/>
       <c r="F18" s="8" t="n">
-        <v>1710200.73</v>
+        <v>1724429.81</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>-9504.85</v>
+        <v>4724.23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>